<commit_message>
Correct BUR500 as Burlington server, not Magnolia
SS-BUR500NSV maps to Burlington Cathedral Doored Server (BUR500NSV).
Refresh Burlington images/copy and note that live McCabe currently
mislabels this SKU as Magnolia; Magnolia servers use MM520*.

Co-authored-by: emcc10 <emcc10@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/imports/steve-silver-volusion/steve_silver_game_dining_server_import.xlsx
+++ b/docs/imports/steve-silver-volusion/steve_silver_game_dining_server_import.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4787,6 +4787,68 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SS-BUR500NSV</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Burlington Cathedral Doored Server</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>A masterpiece of versatility and style, the Burlington Server reveals a world of display possibilities behind beautiful Cathedral glass doors. Hand-stained in a striking cocoa finish with a contrasting black interior, this cabinet features adjustable shelves and hidden cable management for a seamless transition from a dining room sideboard, to a living room entertainment center, or even a stunning hallway console 
+ The clean lines and modern style of the Burlington Server adds elegance, sophistication and storage to any room in a home.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>• Crafted from Oak veneers, Asian hardwood solids and engineered woods
+• Wire Escape back allows this cabinet to double as a media console
+• Cathedral glass door fronts offer a beautiful display area or excellent remote access  for electronics
+• Contrasting black interior beautifully accents the interior with the contrasting cocoa finished exterior
+• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+• Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
+• With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
+• The wood is hand-stained in a natural multi-step cocoa finish with black  interior to highlight the interior of the case while offering a beautiful contrast</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>BUR500NSV</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>https://stevesilver.com/product/burlington-cathedral-doored-server/</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>SS-BUR500NSV-1.jpg;SS-BUR500NSV-altview1.jpg;SS-BUR500NSV-altview2.jpg;SS-BUR500NSV-altview3.jpg;SS-BUR500NSV-altview4.jpg;SS-BUR500NSV-altview5.jpg;SS-BUR500NSV-altview6.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5463,7 +5525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9245,6 +9307,68 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SS-BUR500NSV</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Burlington Cathedral Doored Server</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>A masterpiece of versatility and style, the Burlington Server reveals a world of display possibilities behind beautiful Cathedral glass doors. Hand-stained in a striking cocoa finish with a contrasting black interior, this cabinet features adjustable shelves and hidden cable management for a seamless transition from a dining room sideboard, to a living room entertainment center, or even a stunning hallway console 
+ The clean lines and modern style of the Burlington Server adds elegance, sophistication and storage to any room in a home.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>• Crafted from Oak veneers, Asian hardwood solids and engineered woods
+• Wire Escape back allows this cabinet to double as a media console
+• Cathedral glass door fronts offer a beautiful display area or excellent remote access  for electronics
+• Contrasting black interior beautifully accents the interior with the contrasting cocoa finished exterior
+• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+• Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
+• With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
+• The wood is hand-stained in a natural multi-step cocoa finish with black  interior to highlight the interior of the case while offering a beautiful contrast</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>BUR500NSV</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>https://stevesilver.com/product/burlington-cathedral-doored-server/</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>SS-BUR500NSV-1.jpg;SS-BUR500NSV-altview1.jpg;SS-BUR500NSV-altview2.jpg;SS-BUR500NSV-altview3.jpg;SS-BUR500NSV-altview4.jpg;SS-BUR500NSV-altview5.jpg;SS-BUR500NSV-altview6.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9256,7 +9380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9289,7 +9413,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Magnolia Cathedral Doored Server, Black</t>
+          <t>Burlington Cathedral Doored Server</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -9299,51 +9423,95 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Already on site (cat 217). Primary hero often uses -2T; ensure SS-BUR500NSV-1.jpg is present. Description OK but should use stevesilver.com short description + techspecs bullet format for import consistency.</t>
+          <t>CORRECT: BUR500 = Burlington (vendor SKU BUR500NSV). Live McCabe currently mislabels this code as Magnolia — rename title/description to Burlington and use stevesilver.com Burlington copy. Images refreshed from Burlington product page (not Magnolia MM520*).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SS-AUB500SV</t>
+          <t>SS-MM520KSV</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Auburn Server (listed; Aubrey group)</t>
+          <t>Magnolia Cathedral Doored Server, Black</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Already on site as SS-AUB500SV but copy looks wrong (mentions expanding table). Replace productdescription/techspecs from Aubrey Server Black page; upload missing -1.jpg (altviews exist). Confirm naming: Auburn vs Aubrey.</t>
+          <t>Magnolia server uses MM520* SKUs (not BUR500). Import as SS-MM520KSV. Do not map Magnolia images onto SS-BUR500NSV.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>SS-AUB500SV</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Auburn/Aubrey Server (on site)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Already on site. Title says Auburn; Steve Silver listing is Aubrey Server Black (SS-ABR500KSV). Current description incorrectly mentions expanding table — replace with Aubrey server copy. Images available under SS-ABR500KSV / synced to SS-AUB500SV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>KARINA-SIDEBOARD</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Karina Sideboard</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Already on site. Prefer SS- style code if re-importing; images present.</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Already on site. Not Burlington/Magnolia. Optional: rename to SS- style code on re-import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SS-ABR500KSV</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Aubrey Server, Black (import row)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Correct Aubrey server SKU/format. Use to replace/fix SS-AUB500SV content, or import as new and retire SS-AUB500SV.</t>
         </is>
       </c>
     </row>

</xml_diff>